<commit_message>
fix: TikTok field, updated queue text, mobile button padding
- Replaced Endereco field with TikTok (@ do usuario) in registration form
- POST sends tiktok field to Google Sheets
- Updated PHASE 2 queue text: criador de videos, 12h wait time
- Added pb-20 to action buttons and queue view for mobile dock overlap
- Updated apps-script.js and Excel file column D header

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UpShopee_Cadastros.xlsx
+++ b/UpShopee_Cadastros.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cadastros Vídeo IA" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cadastros Vídeo IA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Instruções" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cadastros Vídeo IA'!$A$1:$G$1</definedName>
@@ -513,7 +513,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Endereço</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">

</xml_diff>